<commit_message>
feat: LLM-based job title declension via OpenRouter
- Add llm_declension.py service using gpt-4o-mini via OpenRouter
- Replace pymorphy3 with LLM for accurate job title declension
- Add retry logic with exponential backoff for rate limits
- Combine tables: 127 + 127 = 254 records total
- Requires OPENROUTER_API_KEY in .env
</commit_message>
<xml_diff>
--- a/word_templates/primer_tablicy.xlsx
+++ b/word_templates/primer_tablicy.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Телеграммы" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E128"/>
+  <dimension ref="A1:E255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3872,6 +3872,3435 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Правительство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Мантуров Денис Валентинович</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Первый заместитель Председателя Правительства</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>103274, Москва, Краснопресненская набережная, дом 2, строение 2</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Правительство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Голикова Татьяна Алексеевна</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Заместитель Председателя Правительства</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>103274, Москва, Краснопресненская набережная, дом 2, строение 2</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Правительство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Оверчук Алексей Логвинович</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Заместитель Председателя Правительства</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>103274, Москва, Краснопресненская набережная, дом 2, строение 2</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Правительство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Патрушев Дмитрий Николаевич</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Заместитель Председателя Правительства</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>103274, Москва, Краснопресненская набережная, дом 2, строение 2</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Правительство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Савельев Виталий Геннадьевич</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Заместитель Председателя Правительства</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>103274, Москва, Краснопресненская набережная, дом 2, строение 2</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Правительство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Трутнев Юрий Петрович</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Заместитель Председателя Правительства</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>103274, Москва, Краснопресненская набережная, дом 2, строение 2</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Правительство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Хуснуллин Марат Шакирзянович</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Заместитель Председателя Правительства</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>103274, Москва, Краснопресненская набережная, дом 2, строение 2</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Правительство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Чернышенко Дмитрий Николаевич</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Заместитель Председателя Правительства</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>103274, Москва, Краснопресненская набережная, дом 2, строение 2</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Правительство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Новак Александр Валентинович</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Заместитель Председателя Правительства</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>103274, Москва, Краснопресненская набережная, дом 2, строение 2</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Правительство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Шеменев Виталий Владимирович</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>начальник секретариата Заместителя Председателя Правительства Российской Федерации</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>103274, Москва, Краснопресненская набережная, дом 2, строение 2</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Правительство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Григоренко Дмитрий Юрьевич</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Заместитель Председателя Правительства Российской Федерации – Руководитель Аппарата Правительства Российской Федерации</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>103274, Москва, Краснопресненская набережная, дом 2, строение 2</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Правительство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Левин Леонид Леонидович</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Первый заместитель Руководителя Аппарата Правительства Российской Федерации</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>103274, Москва, Краснопресненская набережная, дом 2, строение 2</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Правительство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Сидоренко Валерий Валерьевич</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Первый заместитель Руководителя Аппарата Правительства Российской Федерации</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>103274, Москва, Краснопресненская набережная, дом 2, строение 2</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Правительство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Трунин Илья Вячеславович</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Заместитель Руководителя Аппарата Правительства</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>103274, Москва, Краснопресненская набережная, дом 2, строение 2</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Правительство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Уваров Алексей Константинович</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Заместитель Руководителя Аппарата Правительства</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>103274, Москва, Краснопресненская набережная, дом 2, строение 2</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Правительство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Мещеряков Анатолий Анатольевич</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>директор департамента транспорта Правительства Российской Федерации</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>103274, Москва, Краснопресненская набережная, дом 2, строение 2</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Правительство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Иванова Светлана Владимировна</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Директор департамента строительства</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>103274, Москва, Краснопресненская набережная, дом 2, строение 2</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Министрество труда Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Котяков Антон Олегович</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Министр</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>127994, Г. МОСКВА, УЛ. ИЛЬИНКА, 21</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Министрество труда Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Баталина Ольга Юрьевна</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Первый заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>127994, Г. МОСКВА, УЛ. ИЛЬИНКА, 21</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Министрество труда Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Пудов Андрей Николаевич</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Статс-секретарь — заместитель министра</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>127994, Г. МОСКВА, УЛ. ИЛЬИНКА, 21</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Министрество труда Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Абдулхалимов Магомед Султанович</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Заместитель министра</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>127994, Г. МОСКВА, УЛ. ИЛЬИНКА, 21</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Социальный фонд России</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Чирков Сергей Александрович</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Председатель</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>119991, г. Москва, ул. Шаболовка, д. 4 стр. 1</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Министерство финансов Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Силуанов Антон Германович</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Министр</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>109097, Москва, Ильинка, д.9</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Министерство финансов Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Окладникова Ирина Андреевна</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Первый заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>109097, Москва, Ильинка, д.9</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Министерство финансов Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Сазанов Алексей Валерьевич</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Статс-секретарь - заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>109097, Москва, Ильинка, д.9</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Министерство финансов Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Бегчин Николай Аркадьевич</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>109097, Москва, Ильинка, д.9</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Министерство финансов Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Кадочников Павел Анатольевич</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>109097, Москва, Ильинка, д.9</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Министерство финансов Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Колычев Владимир Владимирович</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>109097, Москва, Ильинка, д.9</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Министерство финансов Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Липаев Алексей Анатольевич</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>109097, Москва, Ильинка, д.9</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Министерство финансов Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Моисеев Алексей Владимирович</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>109097, Москва, Ильинка, д.9</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Министерство финансов Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Чебесков Иван Александрович</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>109097, Москва, Ильинка, д.9</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Министерство финансов Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Яковлева Елена Павловна</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>109097, Москва, Ильинка, д.9</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Министерство финансов Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Раймхен Екатерина Александровна</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Департамент бюджетной политики в сфере транспорта, дорожного хозяйства, экологии и природопользования , заместитель директора</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>109097, Москва, Ильинка, д.9</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Федеральная налоговая служба Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Егоров Даниил Вячеславович</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Руководитель Федеральной налоговой службы</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>127381, г. Москва, ул. Неглинная, д. 23</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Федеральная налоговая служба Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Бациев Виктор Валентинович</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Заместитель руководителя</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>127381, г. Москва, ул. Неглинная, д. 23</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Федеральная налоговая служба Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Бондарчук Светлана Леонидовна</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Заместитель руководителя</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>127381, г. Москва, ул. Неглинная, д. 23</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Федеральная налоговая служба Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Бударин Андрей Владимирович</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Заместитель руководителя</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>127381, г. Москва, ул. Неглинная, д. 23</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Федеральная налоговая служба Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Егоричев Александр Валерьевич</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Заместитель руководителя</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>127381, г. Москва, ул. Неглинная, д. 23</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Федеральная налоговая служба Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Колесников Виталий Григорьевич</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>Заместитель руководителя</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>127381, г. Москва, ул. Неглинная, д. 23</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Федеральная налоговая служба Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Петрушин Андрей Станиславович</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>заместитель руководителя</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>127381, г. Москва, ул. Неглинная, д. 23</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Федеральная налоговая служба Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Сатин Дмитрий Станиславович</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Заместитель руководителя</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>127381, г. Москва, ул. Неглинная, д. 23</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Федеральная налоговая служба Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Чекмышев Константин Николаевич</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Заместитель руководителя</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>127381, г. Москва, ул. Неглинная, д. 23</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Федеральная налоговая служба Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Шепелева Юлия Вячеславовна</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Заместитель руководителя</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>127381, г. Москва, ул. Неглинная, д. 23</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Федеральная налоговая служба Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Шиналиев Тимур Николаевич</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Заместитель руководителя</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>127381, г. Москва, ул. Неглинная, д. 23</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Федеральное казначейство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Артюхин Роман Евгеньевич</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Руководитель</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>101000, г. Москва, Большой Златоустинский пер., д. 6, стр. 1</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Федеральное казначейство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Катамадзе Анна Теймуразовна</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Заместитель руководителя</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>101000, г. Москва, Большой Златоустинский пер., д. 6, стр. 1</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Федеральное казначейство Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Горина Наталия Михайловна</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>Заместитель руководителя</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>101000, г. Москва, Большой Златоустинский пер., д. 6, стр. 1</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Федеральная служба по надзору за правами потребителей и благополучию населения Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Попова Анна Юрьевна</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Руководитель</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>127994, г. Москва, Вадковский переулок, дом 18, строение 5</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Счетная палата</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Ковальчук Борис Юрьевич</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Председатель</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>119121, Г. МОСКВА, УЛ. ЗУБОВСКАЯ, Д. 2</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Счетная палата</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Изотова Галина Сергеевна</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>заместитель Председателя Счётной палаты РФ</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>119121, Г. МОСКВА, УЛ. ЗУБОВСКАЯ, Д. 2</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Набиуллина Эльвира Сахипзадовна</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Председатель Центрального банка Российской Федерации</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Симановский Алексей Юрьевич</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>советник Председателя, «Заслуженный экономист Российской Федерации», член Совета директоров ЦБ</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Тулин Дмитрий Владиславович</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Первый заместитель Председателя</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Полякова Ольга Васильевна</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Заместитель Председателя</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Любомудров Максим Германович</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>директор Департамента надзора за системно значимыми кредитными организациями Банка России</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Лунёв Александр Валерьевич</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>руководитель Службы текущего банковского надзора Банка России</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Шабля Богдан Александрович</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>руководитель Службы финансового монитортинга и валютного контроля</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Данилов Александр Сергеевич</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>директор Департамента банковского регулирования и аналитики Банка России</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Бакина Алла Станиславовна</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>директор Департамента национальной платежной системы Банка России</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Чистюхин Владимир Викторович</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Первый заместитель Председателя</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Ковригин Михаил Анатольевич</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>директор Департамента организации международных расчетов</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Тяжельникова Людмила Александровна</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Директор Департамента допуска и прекращения деятельности финансовых организаций</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Белов Сергей Владимирович</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Заместитель Председателя</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Заботкин Алексей Борисович</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Заместитель Председателя</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Кахруманова Зульфия Нукербековна</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Заместитель Председателя</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Попов Андрей Анатольевич</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>начальник Волго-Вятского главного управления Центрального банка Российской Федерации.</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>603008, г. Нижний Новгород, ул. Большая Покровская, 26</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Гузнов Алексей Геннадьевич</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Статс-секретарь - Заместитель Председателя</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Зубарев Герман Александрович</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Заместитель Председателя</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Габуния Филипп Георгиевич</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Заместитель Председателя</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Данилова Елизавета Олеговна</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>директор Департамента финансовой стабильности Банка России, Член Совета директоров Банка России</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Казарин Валерий Сергеевич</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>заместитель председателя</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Дымов Александр Петрович</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Руководитель Службы анализа рисков Банка России</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Кружалов Андрей Васильевич</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Заместитель Председателя</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Горегляд Валерий Павлович</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Главный аудитор</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Каштуров Александр Владимирович</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>директор Департамента операций на финансовых рынках</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Мамута Михаил Валерьевич</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Руководитель Службы по защите прав потребителей и обеспечению доступности финансовых услуг</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Рыклина Марина Владимировна</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Директор Департамента по связям с общественностью</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Мечкова Галина Владимировна</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Руководитель Аппарата</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Тихонова Татьяна Адольфовна</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>директор Департамента кадровой политики Банка России</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>107016, Москва, ул. Неглинная, д. 12</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Центральный банк Российской Федерации</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Марданов Рустэм Хабибович</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>начальник ГУ Банка России по Центральному федеральному округу</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>115035, г. Москва, ул. Балчуг, 2</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Маркеева О.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>МИД</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Бутин Сергей Владимирович</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Первый заместитель Министра иностранных дел Российской Федерации</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>119200, г. Москва, Смоленская-Сенная площадь, д. 32/34</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>МИД</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Галузин Михаил Юрьевич</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>119200, г. Москва, Смоленская-Сенная площадь, д. 32/34</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>МИД</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Панкин Александр Анатольевич</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>119200, г. Москва, Смоленская-Сенная площадь, д. 32/34</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>МИД</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Руденко Андрей Юрьевич</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>119200, г. Москва, Смоленская-Сенная площадь, д. 32/34</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>МИД</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Рябков Сергей Алексеевич</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Заместитель Министра - Латинская Америка</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>119200, г. Москва, Смоленская-Сенная площадь, д. 32/34</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>МИД</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Островский Алексей Владимирович</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Генеральный директор Министерства иностранных дел Российской Федерации</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>119200, г. Москва, Смоленская-Сенная площадь, д. 32/34</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>МИД</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Лысиков Андрей Викторович</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Руководитель Валютно-финансового департамента</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>119200, г. Москва, Смоленская-Сенная площадь, д. 32/34</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>МИД</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Дробинин Алексей Юрьевич</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Директор департамента внешнеполитического планирования</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>119200, г. Москва, Смоленская-Сенная площадь, д. 32/34</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>МИД</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Воробьева Людмила Георгиевна</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Директор Третьего департамента Азии</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>119200, г. Москва, Смоленская-Сенная площадь, д. 32/34</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>МИД</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Стерник Александр Вадимович</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Директор Третьего департамента стран СНГ МИД России</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>119200, г. Москва, Смоленская-Сенная площадь, д. 32/34</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>МИД</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Щетинин Александр Валентинович</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Директор Латиноамериканского департамента МИД России</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>119200, г. Москва, Смоленская-Сенная площадь, д. 32/34</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>МИД</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Кинщак Александр Александрович</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Директор Департамента Ближнего Востока и Северной Африки МИД России</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>119200, г. Москва, Смоленская-Сенная площадь, д. 32/34</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>МИД</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Башкин Анатолий Геннадьевич</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Директор департамента Африки</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>119200, г. Москва, Смоленская-Сенная площадь, д. 32/34</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>МИД</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Довгаленко Татьяна Евгеньевна</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Директор Департамента партнерства с Африкой</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>119200, г. Москва, Смоленская-Сенная площадь, д. 32/34</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Минобрнауки</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Фальков Валерий Николаевич</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Министр</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>125993, г. Москва, Тверская ул., д. 11</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Минобрнауки</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Афанасьев Дмитрий Владимирович</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Заместитель министра</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>125993, г. Москва, Тверская ул., д. 11</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Минобрнауки</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Гатиятов Айрат Ринатович</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>125993, г. Москва, Тверская ул., д. 11</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Минобрнауки</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Петрова Ольга Викторовна</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>125993, г. Москва, Тверская ул., д. 11</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Минобрнауки</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Секиринский Денис Сергеевич</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>125993, г. Москва, Тверская ул., д. 11</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Рослесхоз</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Советников Иван Васильевич</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Руководитель</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>115184, Россия, Москва, Пятницкая улица, дом 59/19</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Минпросвещения</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Кравцов Сергей Сергеевич</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Министр</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>115093, г. Москва, ул. Люсиновская, д. 51</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Минпросвещения</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Бугаев Александр Вячеславович</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>Первый заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>115093, г. Москва, ул. Люсиновская, д. 51</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Минсельхоз</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Лут Оксана Николаевна</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Министр</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>107139, г. Москва, Орликов переулок, д. 1/11</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Минсельхоз</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Фастова Елена Владимировна</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Первый заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>107139, г. Москва, Орликов переулок, д. 1/11</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Минсельхоз</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Афонина Марина Игоревна</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>107139, г. Москва, Орликов переулок, д. 1/11</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Росреестр</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Скуфинский Олег Александрович</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Руководитель</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>101000, Москва, Чистопрудный бульвар, д. 6/19, стр. 1</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Росреестр</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Бутовецкий Алексей Игоревич</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Статс-секретарь - заместитель руководителя</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>101000, Москва, Чистопрудный бульвар, д. 6/19, стр. 1</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>Бакулин Э.</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Минвостокразвития</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Чекунков Алексей Олегович</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Министр</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>119121, г. Москва, ул. Бурденко, д. 14</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Григорьева Е.</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Минздрав</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Мурашко Михаил Альбертович</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Министр</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>127994, ГСП-4, г. Москва, Рахмановский переулок, д. 3.</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Минздрав</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Фисенко Виктор Сергеевич</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Первый заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>127994, ГСП-4, г. Москва, Рахмановский переулок, д. 3.</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Минздрав</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Зеленский Владимир Анатольевич</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>Первый заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>127994, ГСП-4, г. Москва, Рахмановский переулок, д. 3.</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Минздрав</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Салагай Олег Олегович</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Статс-секретарь - Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>127994, ГСП-4, г. Москва, Рахмановский переулок, д. 3.</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Минздрав</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Сибирякова Наталья Витальевна</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>127994, ГСП-4, г. Москва, Рахмановский переулок, д. 3.</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Минздрав</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Ваньков Вадим Валерьевич</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>127994, ГСП-4, г. Москва, Рахмановский переулок, д. 3.</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Минздрав</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Глаголев Сергей Владимирович</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>127994, ГСП-4, г. Москва, Рахмановский переулок, д. 3.</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Минздрав</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Камкин Евгений Геннадьевич</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>127994, ГСП-4, г. Москва, Рахмановский переулок, д. 3.</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Минздрав</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Котова Евгения Григорьевна</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>127994, ГСП-4, г. Москва, Рахмановский переулок, д. 3.</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Минздрав</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Плутницкий Андрей Николаевич</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>127994, ГСП-4, г. Москва, Рахмановский переулок, д. 3.</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Минздрав</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Семёнова Татьяна Владимировна</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>127994, ГСП-4, г. Москва, Рахмановский переулок, д. 3.</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Минприроды</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Козлов Александр Александрович</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Министр</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>127994, ГСП-4, г. Москва, Рахмановский переулок, д. 3.</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Минприроды</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Цыганов Константин Анатольевич</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Первый заместитель</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>125993, г. Москва, ул. Большая Грузинская, 4/6</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Минприроды</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Тетенькин Дмитрий Дмитриевич</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Заместитель Министра</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>125993, г. Москва, ул. Большая Грузинская, 4/6</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Росстат</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Галкин Сергей Сергеевич</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Руководитель</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>107450, Россия, Москва, ул. Мясницкая, д. 39, стр. 1.</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Роспатент</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Зубов Юрий Сергеевич</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Руководитель</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>121059, г. Москва, Бережковская набережная, д. 30, корп. 1</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>ФАС</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Шаскольский Максим Алексеевич</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Руководитель</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>125993, г. Москва, ул. Садовая-Кудринская, д. 11, Д-242, ГСП-3</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>ФАС</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Пузыревский Сергей Анатольевич</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Статс-секретарь - заместитель руководителя</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>125993, г. Москва, ул. Садовая-Кудринская, д. 11, Д-242, ГСП-3</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Росархив</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Серегин Алексей Юрьевич</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>заместитель руководителя</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>115035, г. Москва, Софийская набережная, д. 34, стр. 1</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Червяк И.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>